<commit_message>
Support new Forms xlsx schema; widen card left column
- parseStargrams: map new column names (Your full name, long recipient header, Stargram 2 SKIP-suffix); normalize whitespace in row keys so NBSPs from Forms exports don't break lookups
- test-stargrams.xlsx: regenerated to match new schema (35 cols, Stargrams 1-7)
- StargramCard: left info column 160px -> 220px

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-stargrams.xlsx
+++ b/test-stargrams.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:AI21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,49 +413,97 @@
         <v>Email</v>
       </c>
       <c r="E1" t="str">
-        <v>Your name</v>
+        <v>Name</v>
       </c>
       <c r="F1" t="str">
+        <v>Your full name</v>
+      </c>
+      <c r="G1" t="str">
         <v>Your email address</v>
       </c>
-      <c r="G1" t="str">
-        <v>Stargram Recipient</v>
-      </c>
       <c r="H1" t="str">
+        <v>Stargram recipient (MUST be a student in the cast, crew or orchestra of Footloose)</v>
+      </c>
+      <c r="I1" t="str">
         <v>Do they have any allergies?</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Pick a show</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Pick your Stargram treat</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Stargram message</v>
       </c>
-      <c r="L1" t="str">
-        <v>Do you want to order more?</v>
-      </c>
       <c r="M1" t="str">
-        <v>Stargram 2 - Show Date</v>
+        <v>Stargram 2 - Show Date (SKIP if you only want to buy one Stargram for this student)</v>
       </c>
       <c r="N1" t="str">
-        <v>Stargram 2 - Treat Option</v>
+        <v>Stargram 2 - Treat Option (SKIP if you only want to buy one Stargram for this student)</v>
       </c>
       <c r="O1" t="str">
-        <v>Stargram 2 - Message</v>
+        <v>Stargram 2 - Message (SKIP if you only want to buy one Stargram for this student)</v>
       </c>
       <c r="P1" t="str">
-        <v>Do you want to order more?2</v>
+        <v>Do you want to order another Stargram for this student? (this question is REQUIRED)</v>
       </c>
       <c r="Q1" t="str">
+        <v>Stargram 3 - Show Date</v>
+      </c>
+      <c r="R1" t="str">
         <v>Stargram 3 - Treat Option</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Stargram 3 - Message</v>
       </c>
-      <c r="S1" t="str">
-        <v>Do you want to order more?3</v>
+      <c r="T1" t="str">
+        <v>Do you want to order another Stargram for this student?</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Stargram 4 - Show Date</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Stargram 4 - Treat Option</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Stargram 4 - Message</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Do you want to order another Stargram for this student?2</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>Stargram 5 - Show Date</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Stargram 5 - Treat Option</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Stargram 5 - Message</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>Do you want to order another Stargram for this student?3</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>Stargram 6 - Show Date</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Stargram 6 - Treat Option</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>Stargram 6 - Message</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Do you want to order another Stargram for this student?4</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Stargram 7 - Show Date</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>Stargram 7 - Treat Option</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>Stargram 7 - Message</v>
       </c>
     </row>
     <row r="2">
@@ -472,28 +520,97 @@
         <v>anonymous</v>
       </c>
       <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
         <v>Maria Lopez</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Jake Thompson</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>no</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Fri, Mar 20 - 7pm</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>Chocolate candy</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>Break a leg tonight! So proud of you!</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
         <v>No</v>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+      <c r="AC2" t="str">
+        <v/>
+      </c>
+      <c r="AD2" t="str">
+        <v/>
+      </c>
+      <c r="AE2" t="str">
+        <v/>
+      </c>
+      <c r="AF2" t="str">
+        <v/>
+      </c>
+      <c r="AG2" t="str">
+        <v/>
+      </c>
+      <c r="AH2" t="str">
+        <v/>
+      </c>
+      <c r="AI2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -510,28 +627,97 @@
         <v>anonymous</v>
       </c>
       <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
         <v>David Chen</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Sophie Williams</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>Peanuts</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>Fri, Mar 20 - 7pm</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Gummy bears</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>You are going to be amazing up there. We love you!</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
         <v>No</v>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+      <c r="AC3" t="str">
+        <v/>
+      </c>
+      <c r="AD3" t="str">
+        <v/>
+      </c>
+      <c r="AE3" t="str">
+        <v/>
+      </c>
+      <c r="AF3" t="str">
+        <v/>
+      </c>
+      <c r="AG3" t="str">
+        <v/>
+      </c>
+      <c r="AH3" t="str">
+        <v/>
+      </c>
+      <c r="AI3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -548,28 +734,97 @@
         <v>anonymous</v>
       </c>
       <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
         <v>Grandma Rose</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Ethan Park</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>no</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Sat, Mar 21 - 2pm</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>Lollipop</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>My little star! Grandma is watching from the front row!</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
         <v>No</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+      <c r="AC4" t="str">
+        <v/>
+      </c>
+      <c r="AD4" t="str">
+        <v/>
+      </c>
+      <c r="AE4" t="str">
+        <v/>
+      </c>
+      <c r="AF4" t="str">
+        <v/>
+      </c>
+      <c r="AG4" t="str">
+        <v/>
+      </c>
+      <c r="AH4" t="str">
+        <v/>
+      </c>
+      <c r="AI4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -586,28 +841,97 @@
         <v>anonymous</v>
       </c>
       <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v>The Nguyen Family</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>Lily Nguyen</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>Dairy</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>Sat, Mar 21 - 2pm</v>
       </c>
-      <c r="J5" t="str">
+      <c r="K5" t="str">
         <v>Chocolate candy</v>
       </c>
-      <c r="K5" t="str">
+      <c r="L5" t="str">
         <v>We are all here cheering for you. Shine bright!</v>
       </c>
-      <c r="L5" t="str">
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
         <v>No</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5" t="str">
+        <v/>
+      </c>
+      <c r="AB5" t="str">
+        <v/>
+      </c>
+      <c r="AC5" t="str">
+        <v/>
+      </c>
+      <c r="AD5" t="str">
+        <v/>
+      </c>
+      <c r="AE5" t="str">
+        <v/>
+      </c>
+      <c r="AF5" t="str">
+        <v/>
+      </c>
+      <c r="AG5" t="str">
+        <v/>
+      </c>
+      <c r="AH5" t="str">
+        <v/>
+      </c>
+      <c r="AI5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -624,28 +948,97 @@
         <v>anonymous</v>
       </c>
       <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
         <v>Coach Martinez</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>Whole Cast</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>no</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>Sat, Mar 21 - 7pm</v>
       </c>
-      <c r="J6" t="str">
+      <c r="K6" t="str">
         <v>Gummy bears</v>
       </c>
-      <c r="K6" t="str">
+      <c r="L6" t="str">
         <v>What an incredible group of performers. Enjoy every moment!</v>
       </c>
-      <c r="L6" t="str">
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
         <v>No</v>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
+        <v/>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+      <c r="AA6" t="str">
+        <v/>
+      </c>
+      <c r="AB6" t="str">
+        <v/>
+      </c>
+      <c r="AC6" t="str">
+        <v/>
+      </c>
+      <c r="AD6" t="str">
+        <v/>
+      </c>
+      <c r="AE6" t="str">
+        <v/>
+      </c>
+      <c r="AF6" t="str">
+        <v/>
+      </c>
+      <c r="AG6" t="str">
+        <v/>
+      </c>
+      <c r="AH6" t="str">
+        <v/>
+      </c>
+      <c r="AI6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -662,28 +1055,97 @@
         <v>anonymous</v>
       </c>
       <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
         <v>Auntie Kim</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>Mia Johnson</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>no</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>Sat, Mar 21 - 7pm</v>
       </c>
-      <c r="J7" t="str">
+      <c r="K7" t="str">
         <v>Sour candy</v>
       </c>
-      <c r="K7" t="str">
+      <c r="L7" t="str">
         <v>You were born to be on that stage!</v>
       </c>
-      <c r="L7" t="str">
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
         <v>No</v>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v/>
+      </c>
+      <c r="Y7" t="str">
+        <v/>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
+      </c>
+      <c r="AA7" t="str">
+        <v/>
+      </c>
+      <c r="AB7" t="str">
+        <v/>
+      </c>
+      <c r="AC7" t="str">
+        <v/>
+      </c>
+      <c r="AD7" t="str">
+        <v/>
+      </c>
+      <c r="AE7" t="str">
+        <v/>
+      </c>
+      <c r="AF7" t="str">
+        <v/>
+      </c>
+      <c r="AG7" t="str">
+        <v/>
+      </c>
+      <c r="AH7" t="str">
+        <v/>
+      </c>
+      <c r="AI7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -700,28 +1162,97 @@
         <v>anonymous</v>
       </c>
       <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
         <v>Tyler Brooks</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>Hannah Brooks</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>Tree nuts</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>Fri, Mar 20 - 7pm</v>
       </c>
-      <c r="J8" t="str">
+      <c r="K8" t="str">
         <v>Chocolate candy</v>
       </c>
-      <c r="K8" t="str">
+      <c r="L8" t="str">
         <v>Best sister ever. Knock em dead!</v>
       </c>
-      <c r="L8" t="str">
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
         <v>No</v>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
+      </c>
+      <c r="AA8" t="str">
+        <v/>
+      </c>
+      <c r="AB8" t="str">
+        <v/>
+      </c>
+      <c r="AC8" t="str">
+        <v/>
+      </c>
+      <c r="AD8" t="str">
+        <v/>
+      </c>
+      <c r="AE8" t="str">
+        <v/>
+      </c>
+      <c r="AF8" t="str">
+        <v/>
+      </c>
+      <c r="AG8" t="str">
+        <v/>
+      </c>
+      <c r="AH8" t="str">
+        <v/>
+      </c>
+      <c r="AI8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -738,28 +1269,97 @@
         <v>anonymous</v>
       </c>
       <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
         <v>Mr. and Mrs. Davis</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>Oliver Davis</v>
       </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
         <v>no</v>
       </c>
-      <c r="I9" t="str">
+      <c r="J9" t="str">
         <v>Sat, Mar 21 - 2pm</v>
       </c>
-      <c r="J9" t="str">
+      <c r="K9" t="str">
         <v>Lollipop</v>
       </c>
-      <c r="K9" t="str">
+      <c r="L9" t="str">
         <v>So proud of all your hard work this semester.</v>
       </c>
-      <c r="L9" t="str">
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
         <v>No</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
+      </c>
+      <c r="AA9" t="str">
+        <v/>
+      </c>
+      <c r="AB9" t="str">
+        <v/>
+      </c>
+      <c r="AC9" t="str">
+        <v/>
+      </c>
+      <c r="AD9" t="str">
+        <v/>
+      </c>
+      <c r="AE9" t="str">
+        <v/>
+      </c>
+      <c r="AF9" t="str">
+        <v/>
+      </c>
+      <c r="AG9" t="str">
+        <v/>
+      </c>
+      <c r="AH9" t="str">
+        <v/>
+      </c>
+      <c r="AI9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -776,28 +1376,97 @@
         <v>anonymous</v>
       </c>
       <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
         <v>Jess</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>Chloe Ramirez</v>
       </c>
-      <c r="H10" t="str">
+      <c r="I10" t="str">
         <v>no</v>
       </c>
-      <c r="I10" t="str">
+      <c r="J10" t="str">
         <v>Fri, Mar 20 - 7pm</v>
       </c>
-      <c r="J10" t="str">
+      <c r="K10" t="str">
         <v>Gummy bears</v>
       </c>
-      <c r="K10" t="str">
+      <c r="L10" t="str">
         <v>Best friends forever. You are a STAR!!!!</v>
       </c>
-      <c r="L10" t="str">
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
         <v>No</v>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+      <c r="AA10" t="str">
+        <v/>
+      </c>
+      <c r="AB10" t="str">
+        <v/>
+      </c>
+      <c r="AC10" t="str">
+        <v/>
+      </c>
+      <c r="AD10" t="str">
+        <v/>
+      </c>
+      <c r="AE10" t="str">
+        <v/>
+      </c>
+      <c r="AF10" t="str">
+        <v/>
+      </c>
+      <c r="AG10" t="str">
+        <v/>
+      </c>
+      <c r="AH10" t="str">
+        <v/>
+      </c>
+      <c r="AI10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -814,28 +1483,97 @@
         <v>anonymous</v>
       </c>
       <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
         <v>The Patel Family</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>Arjun Patel</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>Gluten</v>
       </c>
-      <c r="I11" t="str">
+      <c r="J11" t="str">
         <v>Sat, Mar 21 - 7pm</v>
       </c>
-      <c r="J11" t="str">
+      <c r="K11" t="str">
         <v>Chocolate candy</v>
       </c>
-      <c r="K11" t="str">
+      <c r="L11" t="str">
         <v>We drove four hours to see you perform and it is worth every single mile. You have worked so hard this whole year and we could not be more proud of the incredible performer you have become. We love you so much!</v>
       </c>
-      <c r="L11" t="str">
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
         <v>No</v>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v/>
+      </c>
+      <c r="Z11" t="str">
+        <v/>
+      </c>
+      <c r="AA11" t="str">
+        <v/>
+      </c>
+      <c r="AB11" t="str">
+        <v/>
+      </c>
+      <c r="AC11" t="str">
+        <v/>
+      </c>
+      <c r="AD11" t="str">
+        <v/>
+      </c>
+      <c r="AE11" t="str">
+        <v/>
+      </c>
+      <c r="AF11" t="str">
+        <v/>
+      </c>
+      <c r="AG11" t="str">
+        <v/>
+      </c>
+      <c r="AH11" t="str">
+        <v/>
+      </c>
+      <c r="AI11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -852,28 +1590,97 @@
         <v>anonymous</v>
       </c>
       <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
         <v>Mom</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G12" t="str">
+      <c r="H12" t="str">
         <v>Emma Sutton</v>
       </c>
-      <c r="H12" t="str">
+      <c r="I12" t="str">
         <v>no</v>
       </c>
-      <c r="I12" t="str">
+      <c r="J12" t="str">
         <v>Sat, Mar 21 - 2pm</v>
       </c>
-      <c r="J12" t="str">
+      <c r="K12" t="str">
         <v>Sour candy</v>
       </c>
-      <c r="K12" t="str">
+      <c r="L12" t="str">
         <v>My sweet girl, you make me proud every single day.</v>
       </c>
-      <c r="L12" t="str">
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
         <v>No</v>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
+        <v/>
+      </c>
+      <c r="Y12" t="str">
+        <v/>
+      </c>
+      <c r="Z12" t="str">
+        <v/>
+      </c>
+      <c r="AA12" t="str">
+        <v/>
+      </c>
+      <c r="AB12" t="str">
+        <v/>
+      </c>
+      <c r="AC12" t="str">
+        <v/>
+      </c>
+      <c r="AD12" t="str">
+        <v/>
+      </c>
+      <c r="AE12" t="str">
+        <v/>
+      </c>
+      <c r="AF12" t="str">
+        <v/>
+      </c>
+      <c r="AG12" t="str">
+        <v/>
+      </c>
+      <c r="AH12" t="str">
+        <v/>
+      </c>
+      <c r="AI12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -890,28 +1697,97 @@
         <v>anonymous</v>
       </c>
       <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
         <v>Uncle Steve</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G13" t="str">
+      <c r="H13" t="str">
         <v>Noah Garcia</v>
       </c>
-      <c r="H13" t="str">
+      <c r="I13" t="str">
         <v>no</v>
       </c>
-      <c r="I13" t="str">
+      <c r="J13" t="str">
         <v>Fri, Mar 20 - 7pm</v>
       </c>
-      <c r="J13" t="str">
+      <c r="K13" t="str">
         <v>Chocolate candy</v>
       </c>
-      <c r="K13" t="str">
+      <c r="L13" t="str">
         <v>From one performer to another — own that stage!</v>
       </c>
-      <c r="L13" t="str">
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
         <v>No</v>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
+        <v/>
+      </c>
+      <c r="Z13" t="str">
+        <v/>
+      </c>
+      <c r="AA13" t="str">
+        <v/>
+      </c>
+      <c r="AB13" t="str">
+        <v/>
+      </c>
+      <c r="AC13" t="str">
+        <v/>
+      </c>
+      <c r="AD13" t="str">
+        <v/>
+      </c>
+      <c r="AE13" t="str">
+        <v/>
+      </c>
+      <c r="AF13" t="str">
+        <v/>
+      </c>
+      <c r="AG13" t="str">
+        <v/>
+      </c>
+      <c r="AH13" t="str">
+        <v/>
+      </c>
+      <c r="AI13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -928,28 +1804,97 @@
         <v>anonymous</v>
       </c>
       <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
         <v>Sarah and Ben</v>
       </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G14" t="str">
+      <c r="H14" t="str">
         <v>Zoe Mitchell</v>
       </c>
-      <c r="H14" t="str">
+      <c r="I14" t="str">
         <v>Soy</v>
       </c>
-      <c r="I14" t="str">
+      <c r="J14" t="str">
         <v>Sat, Mar 21 - 7pm</v>
       </c>
-      <c r="J14" t="str">
+      <c r="K14" t="str">
         <v>Lollipop</v>
       </c>
-      <c r="K14" t="str">
+      <c r="L14" t="str">
         <v>We cannot wait to see you shine tonight!</v>
       </c>
-      <c r="L14" t="str">
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
         <v>No</v>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14" t="str">
+        <v/>
+      </c>
+      <c r="Z14" t="str">
+        <v/>
+      </c>
+      <c r="AA14" t="str">
+        <v/>
+      </c>
+      <c r="AB14" t="str">
+        <v/>
+      </c>
+      <c r="AC14" t="str">
+        <v/>
+      </c>
+      <c r="AD14" t="str">
+        <v/>
+      </c>
+      <c r="AE14" t="str">
+        <v/>
+      </c>
+      <c r="AF14" t="str">
+        <v/>
+      </c>
+      <c r="AG14" t="str">
+        <v/>
+      </c>
+      <c r="AH14" t="str">
+        <v/>
+      </c>
+      <c r="AI14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -966,28 +1911,97 @@
         <v>anonymous</v>
       </c>
       <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
         <v>Dad</v>
       </c>
-      <c r="F15" t="str">
+      <c r="G15" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G15" t="str">
+      <c r="H15" t="str">
         <v>Lucas Kim</v>
       </c>
-      <c r="H15" t="str">
+      <c r="I15" t="str">
         <v>no</v>
       </c>
-      <c r="I15" t="str">
+      <c r="J15" t="str">
         <v>Sat, Mar 21 - 2pm</v>
       </c>
-      <c r="J15" t="str">
+      <c r="K15" t="str">
         <v>Gummy bears</v>
       </c>
-      <c r="K15" t="str">
+      <c r="L15" t="str">
         <v>Remember: have fun up there. That is what it is all about.</v>
       </c>
-      <c r="L15" t="str">
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
         <v>No</v>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v/>
+      </c>
+      <c r="X15" t="str">
+        <v/>
+      </c>
+      <c r="Y15" t="str">
+        <v/>
+      </c>
+      <c r="Z15" t="str">
+        <v/>
+      </c>
+      <c r="AA15" t="str">
+        <v/>
+      </c>
+      <c r="AB15" t="str">
+        <v/>
+      </c>
+      <c r="AC15" t="str">
+        <v/>
+      </c>
+      <c r="AD15" t="str">
+        <v/>
+      </c>
+      <c r="AE15" t="str">
+        <v/>
+      </c>
+      <c r="AF15" t="str">
+        <v/>
+      </c>
+      <c r="AG15" t="str">
+        <v/>
+      </c>
+      <c r="AH15" t="str">
+        <v/>
+      </c>
+      <c r="AI15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1004,28 +2018,97 @@
         <v>anonymous</v>
       </c>
       <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
         <v>The Entire Kowalski-Beaumont Extended Family Including Grandma Irene</v>
       </c>
-      <c r="F16" t="str">
+      <c r="G16" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G16" t="str">
+      <c r="H16" t="str">
         <v>Alexandria Kowalski-Beaumont III</v>
       </c>
-      <c r="H16" t="str">
+      <c r="I16" t="str">
         <v>Peanuts, tree nuts, shellfish, dairy, soy</v>
       </c>
-      <c r="I16" t="str">
+      <c r="J16" t="str">
         <v>Sat, Mar 21 - 7pm</v>
       </c>
-      <c r="J16" t="str">
+      <c r="K16" t="str">
         <v>Chocolate candy</v>
       </c>
-      <c r="K16" t="str">
+      <c r="L16" t="str">
         <v>We are so incredibly proud of everything you have accomplished this year. From the very first rehearsal all the way to tonight, you have poured your heart and soul into this production and it truly shows. Every single person in this family is cheering for you from the audience tonight. You were born to be on that stage and we cannot wait to see you absolutely shine under those lights. Break a leg, sweetheart! We love you more than words can say!</v>
       </c>
-      <c r="L16" t="str">
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
         <v>No</v>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
+      <c r="W16" t="str">
+        <v/>
+      </c>
+      <c r="X16" t="str">
+        <v/>
+      </c>
+      <c r="Y16" t="str">
+        <v/>
+      </c>
+      <c r="Z16" t="str">
+        <v/>
+      </c>
+      <c r="AA16" t="str">
+        <v/>
+      </c>
+      <c r="AB16" t="str">
+        <v/>
+      </c>
+      <c r="AC16" t="str">
+        <v/>
+      </c>
+      <c r="AD16" t="str">
+        <v/>
+      </c>
+      <c r="AE16" t="str">
+        <v/>
+      </c>
+      <c r="AF16" t="str">
+        <v/>
+      </c>
+      <c r="AG16" t="str">
+        <v/>
+      </c>
+      <c r="AH16" t="str">
+        <v/>
+      </c>
+      <c r="AI16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1042,28 +2125,97 @@
         <v>anonymous</v>
       </c>
       <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
         <v>J</v>
       </c>
-      <c r="F17" t="str">
+      <c r="G17" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G17" t="str">
+      <c r="H17" t="str">
         <v>Z</v>
       </c>
-      <c r="H17" t="str">
+      <c r="I17" t="str">
         <v>no</v>
       </c>
-      <c r="I17" t="str">
+      <c r="J17" t="str">
         <v>Fri, Mar 20 - 7pm</v>
       </c>
-      <c r="J17" t="str">
+      <c r="K17" t="str">
         <v>Lollipop</v>
       </c>
-      <c r="K17" t="str">
+      <c r="L17" t="str">
         <v>!</v>
       </c>
-      <c r="L17" t="str">
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
         <v>No</v>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+      <c r="V17" t="str">
+        <v/>
+      </c>
+      <c r="W17" t="str">
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <v/>
+      </c>
+      <c r="Y17" t="str">
+        <v/>
+      </c>
+      <c r="Z17" t="str">
+        <v/>
+      </c>
+      <c r="AA17" t="str">
+        <v/>
+      </c>
+      <c r="AB17" t="str">
+        <v/>
+      </c>
+      <c r="AC17" t="str">
+        <v/>
+      </c>
+      <c r="AD17" t="str">
+        <v/>
+      </c>
+      <c r="AE17" t="str">
+        <v/>
+      </c>
+      <c r="AF17" t="str">
+        <v/>
+      </c>
+      <c r="AG17" t="str">
+        <v/>
+      </c>
+      <c r="AH17" t="str">
+        <v/>
+      </c>
+      <c r="AI17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1080,28 +2232,97 @@
         <v>anonymous</v>
       </c>
       <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
         <v>Mrs. Bartholomew-Richardson</v>
       </c>
-      <c r="F18" t="str">
+      <c r="G18" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G18" t="str">
+      <c r="H18" t="str">
         <v>The Entire Cast and Crew of the Spring Musical Production</v>
       </c>
-      <c r="H18" t="str">
+      <c r="I18" t="str">
         <v>Gluten, Red dye #40</v>
       </c>
-      <c r="I18" t="str">
+      <c r="J18" t="str">
         <v>Sat, Mar 21 - 2pm &amp; 7pm</v>
       </c>
-      <c r="J18" t="str">
+      <c r="K18" t="str">
         <v>Assorted candy variety pack</v>
       </c>
-      <c r="K18" t="str">
+      <c r="L18" t="str">
         <v>As your drama teacher for the past three years, I have watched each and every one of you grow from nervous newcomers into confident, talented performers. This show represents months of late rehearsals, weekend set-building sessions, countless line run-throughs, and more hard work than anyone in the audience will ever fully appreciate. I want you all to know that regardless of what happens on that stage tonight, you have already succeeded beyond my wildest expectations. This is YOUR moment. Own it. Enjoy every second of it. And remember that the friendships and memories you have made along the way are worth far more than any standing ovation. I love you all. Now go out there and show them what you are made of!</v>
       </c>
-      <c r="L18" t="str">
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
         <v>No</v>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+      <c r="V18" t="str">
+        <v/>
+      </c>
+      <c r="W18" t="str">
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+      <c r="Y18" t="str">
+        <v/>
+      </c>
+      <c r="Z18" t="str">
+        <v/>
+      </c>
+      <c r="AA18" t="str">
+        <v/>
+      </c>
+      <c r="AB18" t="str">
+        <v/>
+      </c>
+      <c r="AC18" t="str">
+        <v/>
+      </c>
+      <c r="AD18" t="str">
+        <v/>
+      </c>
+      <c r="AE18" t="str">
+        <v/>
+      </c>
+      <c r="AF18" t="str">
+        <v/>
+      </c>
+      <c r="AG18" t="str">
+        <v/>
+      </c>
+      <c r="AH18" t="str">
+        <v/>
+      </c>
+      <c r="AI18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1118,28 +2339,97 @@
         <v>anonymous</v>
       </c>
       <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
         <v>Anonymous</v>
       </c>
-      <c r="F19" t="str">
+      <c r="G19" t="str">
         <v>test@example.com</v>
       </c>
-      <c r="G19" t="str">
+      <c r="H19" t="str">
         <v>Mia Johnson</v>
       </c>
-      <c r="H19" t="str">
+      <c r="I19" t="str">
         <v>no</v>
       </c>
-      <c r="I19" t="str">
+      <c r="J19" t="str">
         <v>Fri, Mar 20 - 7pm</v>
       </c>
-      <c r="J19" t="str">
+      <c r="K19" t="str">
         <v>Chocolate candy</v>
       </c>
-      <c r="K19" t="str">
-        <v/>
-      </c>
       <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
         <v>No</v>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+      <c r="V19" t="str">
+        <v/>
+      </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <v/>
+      </c>
+      <c r="Y19" t="str">
+        <v/>
+      </c>
+      <c r="Z19" t="str">
+        <v/>
+      </c>
+      <c r="AA19" t="str">
+        <v/>
+      </c>
+      <c r="AB19" t="str">
+        <v/>
+      </c>
+      <c r="AC19" t="str">
+        <v/>
+      </c>
+      <c r="AD19" t="str">
+        <v/>
+      </c>
+      <c r="AE19" t="str">
+        <v/>
+      </c>
+      <c r="AF19" t="str">
+        <v/>
+      </c>
+      <c r="AG19" t="str">
+        <v/>
+      </c>
+      <c r="AH19" t="str">
+        <v/>
+      </c>
+      <c r="AI19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1156,28 +2446,28 @@
         <v>anonymous</v>
       </c>
       <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
         <v>Karen Wells</v>
       </c>
-      <c r="F20" t="str">
+      <c r="G20" t="str">
         <v>karen@example.com</v>
       </c>
-      <c r="G20" t="str">
+      <c r="H20" t="str">
         <v>Tommy Wells</v>
       </c>
-      <c r="H20" t="str">
+      <c r="I20" t="str">
         <v>no</v>
       </c>
-      <c r="I20" t="str">
+      <c r="J20" t="str">
         <v>Sat, Mar 21 - 2pm</v>
       </c>
-      <c r="J20" t="str">
+      <c r="K20" t="str">
         <v>Chocolate candy</v>
       </c>
-      <c r="K20" t="str">
+      <c r="L20" t="str">
         <v>So proud of you, kiddo!</v>
-      </c>
-      <c r="L20" t="str">
-        <v>Yes</v>
       </c>
       <c r="M20" t="str">
         <v>Sat, Mar 21 - 7pm</v>
@@ -1189,7 +2479,64 @@
         <v>Encore performance! We love you!</v>
       </c>
       <c r="P20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
         <v>No</v>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+      <c r="V20" t="str">
+        <v/>
+      </c>
+      <c r="W20" t="str">
+        <v/>
+      </c>
+      <c r="X20" t="str">
+        <v/>
+      </c>
+      <c r="Y20" t="str">
+        <v/>
+      </c>
+      <c r="Z20" t="str">
+        <v/>
+      </c>
+      <c r="AA20" t="str">
+        <v/>
+      </c>
+      <c r="AB20" t="str">
+        <v/>
+      </c>
+      <c r="AC20" t="str">
+        <v/>
+      </c>
+      <c r="AD20" t="str">
+        <v/>
+      </c>
+      <c r="AE20" t="str">
+        <v/>
+      </c>
+      <c r="AF20" t="str">
+        <v/>
+      </c>
+      <c r="AG20" t="str">
+        <v/>
+      </c>
+      <c r="AH20" t="str">
+        <v/>
+      </c>
+      <c r="AI20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1206,28 +2553,28 @@
         <v>anonymous</v>
       </c>
       <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
         <v>Bob and Linda</v>
       </c>
-      <c r="F21" t="str">
+      <c r="G21" t="str">
         <v>bob@example.com</v>
       </c>
-      <c r="G21" t="str">
+      <c r="H21" t="str">
         <v>Tina Belcher</v>
       </c>
-      <c r="H21" t="str">
+      <c r="I21" t="str">
         <v>Dairy</v>
       </c>
-      <c r="I21" t="str">
+      <c r="J21" t="str">
         <v>Fri, Mar 20 - 7pm</v>
       </c>
-      <c r="J21" t="str">
+      <c r="K21" t="str">
         <v>Sour candy</v>
       </c>
-      <c r="K21" t="str">
+      <c r="L21" t="str">
         <v>Our little star! First show!</v>
-      </c>
-      <c r="L21" t="str">
-        <v>Yes</v>
       </c>
       <c r="M21" t="str">
         <v>Sat, Mar 21 - 2pm</v>
@@ -1242,18 +2589,66 @@
         <v>Yes</v>
       </c>
       <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
         <v>Sour candy</v>
       </c>
-      <c r="R21" t="str">
+      <c r="S21" t="str">
         <v>Final show! Give it everything!</v>
       </c>
-      <c r="S21" t="str">
+      <c r="T21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="U21" t="str">
+        <v/>
+      </c>
+      <c r="V21" t="str">
+        <v/>
+      </c>
+      <c r="W21" t="str">
+        <v/>
+      </c>
+      <c r="X21" t="str">
         <v>No</v>
+      </c>
+      <c r="Y21" t="str">
+        <v/>
+      </c>
+      <c r="Z21" t="str">
+        <v/>
+      </c>
+      <c r="AA21" t="str">
+        <v/>
+      </c>
+      <c r="AB21" t="str">
+        <v/>
+      </c>
+      <c r="AC21" t="str">
+        <v/>
+      </c>
+      <c r="AD21" t="str">
+        <v/>
+      </c>
+      <c r="AE21" t="str">
+        <v/>
+      </c>
+      <c r="AF21" t="str">
+        <v/>
+      </c>
+      <c r="AG21" t="str">
+        <v/>
+      </c>
+      <c r="AH21" t="str">
+        <v/>
+      </c>
+      <c r="AI21" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AI21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>